<commit_message>
feat: align with CSE3066 official rubric - 16 bugs across 5 categories, 13-column Bug Manifest, and Bug_Report tab
</commit_message>
<xml_diff>
--- a/NOP_BAI_DRIVE/Mau_03_Bo_bieu_mau_Kiem_thu.xlsx
+++ b/NOP_BAI_DRIVE/Mau_03_Bo_bieu_mau_Kiem_thu.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Report" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,12 +506,12 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -655,7 +656,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-01)</t>
+          <t>FAIL (SEED-01)</t>
         </is>
       </c>
     </row>
@@ -701,7 +702,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-02)</t>
+          <t>FAIL (SEED-02)</t>
         </is>
       </c>
     </row>
@@ -746,7 +747,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-03)</t>
+          <t>FAIL (SEED-03)</t>
         </is>
       </c>
     </row>
@@ -793,7 +794,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-04)</t>
+          <t>FAIL (SEED-04)</t>
         </is>
       </c>
     </row>
@@ -879,7 +880,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-05)</t>
+          <t>FAIL (SEED-05)</t>
         </is>
       </c>
     </row>
@@ -891,165 +892,164 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
+          <t>Giới hạn giao diện</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Kiểm tra nhập chuỗi số dài hơn 16 số</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Màn hình là 0</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>1. Bấm phím 9 liên tục 25 lần</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>25 số 9</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Giới hạn 16 số hoặc co chữ e-notation</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>FAIL (SEED-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Đổi dấu</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Kiểm tra đổi dấu trên số 0</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Màn hình là 0</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>1. Màn hình là 0 -&gt; Bấm ±</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>±(0)</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Giữ nguyên là 0, căn lề chuẩn</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>FAIL (SEED-07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Nhật ký lịch sử</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Kiểm tra thẻ lịch sử hiển thị biểu thức dài</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Màn hình là 0</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập 123456789 + 987654321 =</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Biểu thức dài</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Bẻ dòng gọn gàng, không vỡ khung</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>FAIL (SEED-08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>TC-11</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
           <t>Kiểm tra nhập liệu</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Kiểm tra nhập nhiều số 0 vô nghĩa ở đầu</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Màn hình là 0</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>1. Bấm 0 ba lần
 2. Bấm 8</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>0008</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Chuẩn hóa thành 8</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>FAIL (BUG-06)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>TC-09</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Giới hạn giao diện</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra nhập chuỗi số dài hơn 16 số</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Màn hình là 0</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>1. Bấm phím 9 liên tục 25 lần</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>25 số 9</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Giới hạn 15 ký tự hoặc co chữ e-notation</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>FAIL (BUG-07)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>TC-10</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Xóa ký tự</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra phím Backspace khi còn 1 số</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Màn hình có số 5</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>1. Bấm phím ⌫</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>5 -&gt; ⌫</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>Màn hình quay về 0</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>FAIL (BUG-08)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>TC-11</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Toán tử liên tiếp</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra thay đổi toán tử giữa chừng</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Màn hình là 0</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>1. Nhập 5 -&gt; Bấm +
-2. Bấm × -&gt; Nhập 2 -&gt; Bấm =</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>5 + × 2</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Toán tử × thay thế +, kết quả là 10</t>
-        </is>
-      </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-09)</t>
+          <t>FAIL (SEED-09)</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-10)</t>
+          <t>FAIL (SEED-10)</t>
         </is>
       </c>
     </row>
@@ -1104,39 +1104,37 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Bộ nhớ tạm</t>
+          <t>Nhãn giao diện</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra nút C không được xóa Memory</t>
+          <t>Kiểm tra tooltip nút C</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Bộ nhớ lưu 50</t>
+          <t>Màn hình chính</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>1. Nhập 50 -&gt; Bấm MS
-2. Nhập 99 -&gt; Bấm C
-3. Bấm MR</t>
+          <t>1. Rê chuột lên nút C</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>MS: 50, C, MR</t>
+          <t>Tooltip nút C</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>MR phục hồi lại số 50</t>
+          <t>Tooltip: Clear Entry</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-11)</t>
+          <t>FAIL (SEED-11)</t>
         </is>
       </c>
     </row>
@@ -1148,39 +1146,37 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Bộ nhớ tạm</t>
+          <t>Hiệu năng CPU</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra nút M- (Memory Subtract)</t>
+          <t>Kiểm tra tính bình phương phản hồi tức thì</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Bộ nhớ lưu 100</t>
+          <t>Màn hình là 0</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>1. Nhập 100 -&gt; MS
-2. Nhập 30 -&gt; M-
-3. Bấm MR</t>
+          <t>1. Nhập 5 -&gt; Bấm x²</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>100 - 30</t>
+          <t>5²</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>MR hiển thị 70</t>
+          <t>Hiển thị 25 ngay lập tức (&lt; 50ms)</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-12)</t>
+          <t>FAIL (SEED-12: Treo &gt; 3s)</t>
         </is>
       </c>
     </row>
@@ -1192,37 +1188,38 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Đổi dấu</t>
+          <t>Giải phóng RAM</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra đổi dấu trên số 0</t>
+          <t>Kiểm tra giải phóng bộ nhớ khi xóa lịch sử</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Màn hình là 0</t>
+          <t>Có lịch sử</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>1. Màn hình là 0 -&gt; Bấm ±</t>
+          <t>1. Tính 1+1=2 -&gt; Bấm Xóa lịch sử
+2. Tính 2+2=4</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>±(0)</t>
+          <t>Clear History</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Giữ nguyên là 0</t>
+          <t>Lịch sử chỉ chứa duy nhất 2+2=4</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-13)</t>
+          <t>FAIL (SEED-13: Rò rỉ RAM)</t>
         </is>
       </c>
     </row>
@@ -1234,38 +1231,37 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Phím Bằng</t>
+          <t>Độ ổn định</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra bấm phím = lặp lại</t>
+          <t>Kiểm tra xóa rỗng rồi bấm tính toán</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Màn hình là 0</t>
+          <t>Màn hình có số 5</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>1. Nhập 5 + 2 = (ra 7)
-2. Bấm tiếp phím =</t>
+          <t>1. Bấm ⌫ -&gt; Bấm + -&gt; Bấm =</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>5 + 2 = =</t>
+          <t>Backspace rỗng</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Tiếp tục cộng 2 thành 9</t>
+          <t>Về 0, không ném lỗi</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-14)</t>
+          <t>FAIL (SEED-14: Crash ứng dụng)</t>
         </is>
       </c>
     </row>
@@ -1277,39 +1273,37 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Nhật ký lịch sử</t>
+          <t>Độ ổn định</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra xóa lịch sử và tính phép mới</t>
+          <t>Kiểm tra bấm chuỗi toán tử bất thường</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Có lịch sử</t>
+          <t>Màn hình là 0</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>1. Tính 1+1=2
-2. Bấm Xóa lịch sử
-3. Tính 2+2=4</t>
+          <t>1. Bấm 8 -&gt; Bấm ÷ -&gt; Bấm × -&gt; Bấm =</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Clear History</t>
+          <t>8 ÷ × =</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Lịch sử chỉ chứa duy nhất 2+2=4</t>
+          <t>Báo lỗi cú pháp nhẹ nhàng</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>FAIL (BUG-15)</t>
+          <t>FAIL (SEED-15: White Screen)</t>
         </is>
       </c>
     </row>
@@ -1321,37 +1315,39 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Bình phương</t>
+          <t>Bộ nhớ tạm</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra hàm tính bình phương</t>
+          <t>Kiểm tra nút M- (Memory Subtract)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Màn hình là 0</t>
+          <t>Bộ nhớ lưu 100</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>1. Nhập 8 -&gt; Bấm x²</t>
+          <t>1. Lưu 100 vào MS
+2. Nhập 30 -&gt; Bấm M-
+3. Bấm MR</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>8²</t>
+          <t>100 - 30</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Hiển thị 64</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>MR hiển thị 70</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>FAIL (SEED-16: Tính nhầm thành cộng)</t>
         </is>
       </c>
     </row>
@@ -1445,4 +1441,876 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BÁO CÁO LỖI PHẦN MỀM (BUG REPORT) - DÀNH CHO TESTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Bug ID</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Loại lỗi (5 nhóm)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Mức nghiêm trọng</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Tiêu đề lỗi</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Các bước tái hiện</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Người báo cáo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>BUG-01</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Sai số dấu phẩy động 0.1 + 0.2 ra 0.30000000000000004</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập 0.1 -&gt; +
+2. Nhập 0.2 -&gt; =</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>0.30000000000000004</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>img_01.png</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>BUG-02</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Cho phép nhập nhiều dấu chấm thập phân 5.2.3</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập 5 -&gt; .
+2. Nhập 2 -&gt; .
+3. Nhập 3</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>5.2.3</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>5.23</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>img_02.png</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>BUG-03</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Chia cho 0 ra Infinity thay vì báo lỗi</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập 9 ÷ 0 =</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Infinity</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Báo lỗi Cannot divide by 0</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>img_03.png</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>BUG-04</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Vi phạm thứ tự ưu tiên BODMAS (2 + 3 * 4 ra 20)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập 2 + 3 × 4 =</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>img_04.png</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>BUG-05</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Căn bậc hai số âm ra NaN</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập -9 -&gt; √</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid Input</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>img_05.png</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>BUG-06</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Tràn màn hình khi nhập quá 16 số</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập liên tục 25 số 9</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Tràn vỡ khung viền</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Tự co cỡ chữ / e-notation</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>img_06.png</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>BUG-07</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Đổi dấu số 0 biến thành -0 và nhảy lệch lề</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>1. Đang là 0 -&gt; Bấm ±</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>-0 và thụt lề trái</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>0 và căn lề phải</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>img_07.png</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>BUG-08</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Thẻ lịch sử vỡ khung khi biểu thức dài</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập phép tính số dài 9 chữ số</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Tràn khung thẻ</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Tự bẻ dòng gọn gàng</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>img_08.png</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>BUG-09</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Cho phép nhiều số 0 vô nghĩa ở đầu (0008)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>1. Bấm 0 ba lần -&gt; Bấm 8</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>0008</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>img_09.png</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>BUG-10</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Sai công thức phần trăm: 100 + 10% ra 100.1</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>1. 100 + 10 % =</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>100.1</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>img_10.png</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>BUG-11</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Tooltip nút C ghi sai thành Clear All Data &amp; Memory</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>1. Rê chuột lên nút C</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Clear All Data &amp; Memory</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Clear Entry</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>img_11.png</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BUG-12</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Đơ lag trình duyệt &gt; 3 giây khi bấm x²</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập 5 -&gt; Bấm x²</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Treo CPU Main Thread &gt; 3.5s</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Phản hồi &lt; 50ms</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>log_perf.png</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BUG-13</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Rò rỉ bộ nhớ RAM khi bấm Xóa lịch sử</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>1. Tính 1+1=2 -&gt; Xóa lịch sử
+2. Tính 2+2=4</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Phép tính cũ bị phục hồi lại</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>RAM được giải phóng</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>log_mem.png</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>BUG-14</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Crash</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Sập ứng dụng khi xóa rỗng rồi bấm tính toán</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>1. Bấm ⌫ xóa sạch -&gt; Bấm + =</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Uncaught TypeError, đơ máy tính</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Trở về 0 an toàn</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>crash_01.png</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>BUG-15</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Crash</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Trắng màn hình khi bấm chuỗi toán tử bất thường</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>1. 8 ÷ × =</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Màn hình trắng xóa Fatal 500</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Báo lỗi cú pháp</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>crash_02.png</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Phạm Văn Quang</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>